<commit_message>
auto: 작업 자동 저장 2026-09-07 08:05
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/results/전달함_팀장님/CI_성적_Vertex_3열비교집계.xlsx
+++ b/eval-runner/orchestrator/results/전달함_팀장님/CI_성적_Vertex_3열비교집계.xlsx
@@ -430,7 +430,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vertex 비교 — 자사 r4 / Vertex 기본값 판 / Vertex 손잡이 판 (같은 시험지 488 · 같은 코퍼스 · 같은 채점기) · 2026-09-04</t>
+          <t>Vertex 비교 — 자사 r4 / Vertex 기본값 판 / Vertex 옵션 변경 판 (같은 시험지 488 · 같은 코퍼스 · 같은 채점기) · 2026-09-04</t>
         </is>
       </c>
     </row>
@@ -453,7 +453,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Vertex 손잡이 판(9/4)</t>
+          <t>Vertex 옵션 변경 판(9/4)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>손잡이 +14.1%p · 자사와 −11.5%p</t>
+          <t>옵션 +14.1%p · 자사와 −11.5%p</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,6 @@
           <t>46 / 104</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -535,7 +534,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>손잡이 판도 3 — 오귀속 2 + 시점 오귀속 1</t>
+          <t>옵션 변경 판도 3 — 오귀속 2 + 시점 오귀속 1</t>
         </is>
       </c>
     </row>
@@ -560,7 +559,6 @@
           <t>37</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -691,7 +689,6 @@
           <t>71.7%</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -714,7 +711,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -791,7 +787,6 @@
           <t>87.7%</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -814,7 +809,6 @@
           <t>0.51s(검색)+0.50s(리랭크)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -839,7 +833,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>손잡이 판: answer API 4.7s</t>
+          <t>옵션 변경 판: answer API 4.7s</t>
         </is>
       </c>
     </row>
@@ -847,7 +841,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>■ 손잡이 판 설정</t>
+          <t>■ 옵션 변경 판 설정</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">

</xml_diff>